<commit_message>
update 2026-09-27 23:53 (plan 2026-09)
</commit_message>
<xml_diff>
--- a/834e3a41b4_Financial_Analysis_2026.xlsx
+++ b/834e3a41b4_Financial_Analysis_2026.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -494,7 +494,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>كشف معاملات البطاقة (12/09/2026 - 17/09/2026)</t>
+          <t>كشف معاملات البطاقة (21/09/2026 - 25/09/2026)</t>
         </is>
       </c>
     </row>
@@ -537,172 +537,81 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>46277</v>
+        <v>46286</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>مصروف</t>
+          <t>وارد</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>ATM - MAADI</t>
+          <t>IBRAHIM SAID ABDEAZI</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>سحب نقدي (ATM)</t>
+          <t>وارد</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>250</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>4750</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>4750</v>
-      </c>
+        <v>1000</v>
+      </c>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>46278</v>
+        <v>46290</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>مصروف</t>
+          <t>وارد</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>OLA ENERGY</t>
+          <t>محمد رفيق حلمى عبدالحمي ب</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>بنزين ووقود</t>
+          <t>وارد</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>180</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>4570</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>4570</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>46279</v>
+        <v>46290</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>وارد</t>
+          <t>مصروف</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>شركة النيل</t>
+          <t>Indriver</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>وارد</t>
+          <t>أخرى (غير مصنف)</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F6" s="5" t="n"/>
+        <v>60</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1057.98</v>
+      </c>
       <c r="G6" s="5" t="n">
-        <v>14570</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>46280</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>مصروف</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>TALABAT</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>مطاعم وتوصيل</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>300</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>14270</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>14270</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>رد مبلغ</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>صيدلة تجريبية يوم 16/9/2026</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>رد مبلغ</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n">
-        <v>14310</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>46282</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>مصروف</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>VODAFONE</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>موبايل وإنترنت</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>600</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>13710</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>13710</v>
+        <v>1057.98</v>
       </c>
     </row>
   </sheetData>
@@ -779,22 +688,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>1330</v>
+        <v>320</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>1290</v>
+        <v>320</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>10000</v>
+        <v>1200</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>8710</v>
+        <v>880</v>
       </c>
     </row>
     <row r="5">
@@ -804,22 +713,22 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1330</v>
+        <v>320</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1290</v>
+        <v>320</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>10000</v>
+        <v>1200</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>8710</v>
+        <v>880</v>
       </c>
     </row>
   </sheetData>
@@ -833,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -874,65 +783,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>موبايل وإنترنت</t>
+          <t>كافيهات وترفيه</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>600</v>
+        <v>255</v>
       </c>
       <c r="D4" t="n">
-        <v>45.1</v>
+        <v>79.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>مطاعم وتوصيل</t>
+          <t>أخرى (غير مصنف)</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="D5" t="n">
-        <v>22.6</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>سحب نقدي (ATM)</t>
+          <t>مطاعم وتوصيل</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>250</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>18.8</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>بنزين ووقود</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="D7" t="n">
-        <v>13.5</v>
+        <v>1.6</v>
       </c>
     </row>
   </sheetData>
@@ -946,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -995,20 +888,20 @@
         <v>1</v>
       </c>
       <c r="B4" s="9" t="n">
-        <v>46282</v>
+        <v>46290</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>VODAFONE</t>
+          <t>CHILLOUT TRUIMPH CAIRO EG</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>موبايل وإنترنت</t>
+          <t>كافيهات وترفيه</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>600</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5">
@@ -1016,20 +909,20 @@
         <v>2</v>
       </c>
       <c r="B5" s="9" t="n">
-        <v>46280</v>
+        <v>46290</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TALABAT</t>
+          <t>Indriver</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>مطاعم وتوصيل</t>
+          <t>أخرى (غير مصنف)</t>
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>300</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -1037,41 +930,20 @@
         <v>3</v>
       </c>
       <c r="B6" s="9" t="n">
-        <v>46277</v>
+        <v>46290</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ATM - MAADI</t>
+          <t>Uber Downtown EG</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>سحب نقدي (ATM)</t>
+          <t>مطاعم وتوصيل</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="9" t="n">
-        <v>46278</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>OLA ENERGY</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>بنزين ووقود</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>180</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1085,7 +957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1120,24 +992,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>شركة النيل</t>
+          <t>IBRAHIM SAID ABDEAZI</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>محمد رفيق حلمى عبدالحمي ب</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n">
-        <v>10000</v>
+      <c r="C6" s="10" t="n">
+        <v>1200</v>
       </c>
     </row>
   </sheetData>
@@ -1162,7 +1047,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>مؤشرات عامة - فترة 12/09/2026 حتى 17/09/2026</t>
+          <t>مؤشرات عامة - فترة 21/09/2026 حتى 25/09/2026</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1075,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
@@ -1201,7 +1086,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
@@ -1212,7 +1097,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1227,11 +1112,11 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>300.0 EGP محاولة فاشلة (لم تخصم)</t>
+          <t>0 EGP محاولة فاشلة (لم تخصم)</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1127,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>1330</v>
+        <v>320</v>
       </c>
       <c r="C8" t="inlineStr"/>
     </row>
@@ -1253,7 +1138,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C9" t="inlineStr"/>
     </row>
@@ -1264,7 +1149,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>1290</v>
+        <v>320</v>
       </c>
       <c r="C10" t="inlineStr"/>
     </row>
@@ -1275,7 +1160,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1290,7 +1175,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>1040</v>
+        <v>320</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
@@ -1301,7 +1186,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>10000</v>
+        <v>1200</v>
       </c>
       <c r="C13" t="inlineStr"/>
     </row>
@@ -1312,7 +1197,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>8710</v>
+        <v>880</v>
       </c>
       <c r="C14" t="inlineStr"/>
     </row>
@@ -1323,7 +1208,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>215</v>
+        <v>64</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
@@ -1334,7 +1219,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>6544.6</v>
+        <v>1948.16</v>
       </c>
       <c r="C16" t="inlineStr"/>
     </row>
@@ -1345,7 +1230,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>5000</v>
+        <v>1117.98</v>
       </c>
       <c r="C17" t="inlineStr"/>
     </row>
@@ -1356,7 +1241,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>13710</v>
+        <v>1057.98</v>
       </c>
       <c r="C18" t="inlineStr"/>
     </row>
@@ -1367,7 +1252,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>13710</v>
+        <v>1057.98</v>
       </c>
       <c r="C19" t="inlineStr"/>
     </row>

</xml_diff>